<commit_message>
Scope the avatar test's voice check to SA English and Afrikaans
Founder decision 2026-10-05: isiZulu, Sesotho and other languages are
deferred to later sprints. Afrikaans voice-check script written in; Piper
and Kokoro have no Afrikaans voice (checked), MMS afr serves the internal
check only (non-commercial), Google Cloud TTS af-ZA or ElevenLabs for a
publishable voice. Sheet, notebook, runbook, kit and prompts updated; the
Local voice gate now reads the Afrikaans column (re-verified pass/fail).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011sciWmQNcts4uDwB8L9SPT
</commit_message>
<xml_diff>
--- a/docs/go-to-market/08_Flux_Loop/Avatar_Test_Run/Avatar_Test_Scoring.xlsx
+++ b/docs/go-to-market/08_Flux_Loop/Avatar_Test_Run/Avatar_Test_Scoring.xlsx
@@ -2138,15 +2138,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2159,7 +2158,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rated by a fluent speaker of each language: natural / OK / poor / not available. Script: Production_Prompts.md §2.</t>
+          <t>South African English and Afrikaans, rated by a fluent speaker: natural / OK / poor / not available. Other languages are deferred to later sprints. Script: Production_Prompts.md §2.</t>
         </is>
       </c>
     </row>
@@ -2176,20 +2175,15 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>isiZulu</t>
+          <t>Afrikaans</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Sesotho</t>
+          <t>Rated by (initials)</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Rated by (initials)</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2198,14 +2192,13 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Higgsfield: ElevenLabs v4</t>
+          <t>Higgsfield: ElevenLabs v4 (supports Afrikaans)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
       <c r="C4" s="4" t="n"/>
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2217,43 +2210,43 @@
       <c r="C5" s="4" t="n"/>
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Higgsfield: Seed Audio</t>
+          <t>Google Cloud Text-to-Speech (af-ZA voices)</t>
         </is>
       </c>
       <c r="B6" s="4" t="n"/>
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Google Cloud Text-to-Speech</t>
+          <t>Meta MMS-TTS afr (Colab; internal check only, non-commercial)</t>
         </is>
       </c>
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="4" t="n"/>
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="4" t="n"/>
-      <c r="F7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Veo (speech in video)</t>
+          <t>Kokoro-82M (Colab; English only)</t>
         </is>
       </c>
       <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>not available</t>
+        </is>
+      </c>
       <c r="D8" s="4" t="n"/>
       <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2265,11 +2258,10 @@
       <c r="C9" s="4" t="n"/>
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="4" t="n"/>
-      <c r="F9" s="4" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="B4:D9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B4:C9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"natural,OK,poor,not available"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3217,15 +3209,15 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>At least one tool rated natural in isiZulu or Sesotho by a fluent speaker</t>
+          <t>At least one tool rated natural in Afrikaans by a fluent speaker</t>
         </is>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIF('Voice check'!$C$4:$D$9,"natural")&amp;" natural rating(s)"</f>
+        <f>COUNTIF('Voice check'!$C$4:$C$9,"natural")&amp;" natural rating(s)"</f>
         <v/>
       </c>
       <c r="D11" s="9">
-        <f>IF(COUNTIF('Voice check'!$C$4:$D$9,"natural")&gt;0,"PASS",IF(COUNTA('Voice check'!$C$4:$D$9)=0,"NEED DATA","FAIL"))</f>
+        <f>IF(COUNTIF('Voice check'!$C$4:$C$9,"natural")&gt;0,"PASS",IF(COUNTA('Voice check'!$C$4:$C$9)=0,"NEED DATA","FAIL"))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Dry run: log business 00 posting (B first, 6 Oct) on the sheet and in the doc
Add fill_dry_run() to the scoring-sheet builder so the FluxMuse record
(A not posted, B posted to TikTok 08:15 and WhatsApp Status 08:20 SAST,
C not filmed) is reproducible; rebuild the sheet; note the actual posting
order and the 72 h measuring point.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011sciWmQNcts4uDwB8L9SPT
</commit_message>
<xml_diff>
--- a/docs/go-to-market/08_Flux_Loop/Avatar_Test_Run/Avatar_Test_Scoring.xlsx
+++ b/docs/go-to-market/08_Flux_Loop/Avatar_Test_Run/Avatar_Test_Scoring.xlsx
@@ -612,7 +612,7 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>C, A, B</t>
+          <t>B first (6 Oct 2026); A, C not posted</t>
         </is>
       </c>
       <c r="L4" s="4" t="n"/>
@@ -1078,19 +1078,45 @@
           <t>A</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F4" s="4" t="n"/>
       <c r="G4" s="4" t="n"/>
       <c r="H4" s="4" t="n"/>
       <c r="I4" s="4" t="n"/>
       <c r="J4" s="4" t="n"/>
-      <c r="K4" s="4" t="n"/>
-      <c r="L4" s="4" t="n"/>
-      <c r="M4" s="4" t="n"/>
-      <c r="N4" s="4" t="n"/>
-      <c r="O4" s="4" t="n"/>
-      <c r="P4" s="4" t="n"/>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>Founder's animated avatar clip (Higgsfield) + Kokoro bf_emma + assemble_video.py; SadTalker/Wav2Lip re-sync failed on CPU</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>Founder: 'better with no avatar'. Lips don't match the words. 1 Higgsfield credit for the Soul image (rand value not known); clip made on the founder's own account.</t>
+        </is>
+      </c>
       <c r="Q4" s="5" t="n">
         <v>0</v>
       </c>
@@ -1110,19 +1136,45 @@
           <t>B</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>6 Oct 2026: TikTok 08:15, WhatsApp Status 08:20 (SAST)</t>
+        </is>
+      </c>
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="4" t="n"/>
       <c r="J5" s="4" t="n"/>
       <c r="K5" s="5" t="n"/>
-      <c r="L5" s="4" t="n"/>
-      <c r="M5" s="4" t="n"/>
-      <c r="N5" s="4" t="n"/>
-      <c r="O5" s="4" t="n"/>
-      <c r="P5" s="4" t="n"/>
+      <c r="L5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>Kokoro-82M bf_emma (Apache 2.0) + assemble_video.py (ffmpeg)</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
+          <t>Posted first, against the planned C, A, B order. Views/conversations/orders due 72 h after post (9 Oct, ~08:20). TikTok posted via Higgsfield connector with 'Your brand' and AI-content labels.</t>
+        </is>
+      </c>
       <c r="Q5" s="5" t="n">
         <v>0</v>
       </c>
@@ -1142,19 +1194,37 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="4" t="n"/>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="4" t="n"/>
       <c r="K6" s="5" t="n"/>
-      <c r="L6" s="4" t="n"/>
-      <c r="M6" s="4" t="n"/>
-      <c r="N6" s="4" t="n"/>
+      <c r="L6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="O6" s="4" t="n"/>
-      <c r="P6" s="4" t="n"/>
+      <c r="P6" s="4" t="inlineStr">
+        <is>
+          <t>Owner didn't film.</t>
+        </is>
+      </c>
       <c r="Q6" s="5" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Dry run: AV00B 72-hour result (0 coded chats, 0 orders) and what it tells us
Logs business 00 format B's 72 h window on the scoring sheet (via
fill_dry_run) and in FluxMuse_Dry_Run.md: no AV00B-coded conversations or
orders; the 15 new chats in the window came from Meta ads. Adds a summary of
what the dry run shows about tracking, cost, Fluxy and reach. Views and
comments still to be filled from the founder's screenshots.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011sciWmQNcts4uDwB8L9SPT
</commit_message>
<xml_diff>
--- a/docs/go-to-market/08_Flux_Loop/Avatar_Test_Run/Avatar_Test_Scoring.xlsx
+++ b/docs/go-to-market/08_Flux_Loop/Avatar_Test_Run/Avatar_Test_Scoring.xlsx
@@ -1152,8 +1152,12 @@
         </is>
       </c>
       <c r="G5" s="4" t="n"/>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="4" t="n"/>
+      <c r="H5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="J5" s="4" t="n"/>
       <c r="K5" s="5" t="n"/>
       <c r="L5" s="4" t="n">
@@ -1172,7 +1176,7 @@
       </c>
       <c r="P5" s="4" t="inlineStr">
         <is>
-          <t>Posted first, against the planned C, A, B order. Views/conversations/orders due 72 h after post (9 Oct, ~08:20). TikTok posted via Higgsfield connector with 'Your brand' and AI-content labels.</t>
+          <t>Posted first, against the planned C, A, B order. 72 h result (to 9 Oct 08:20 SAST): 0 chats with the AV00B code, 0 orders; 15 new FluxMuse chats in the window, none mentioning the video (they came from Meta ads). Views and comments: founder to add from TikTok/Status screenshots. TikTok posted via Higgsfield connector with 'Your brand' and AI-content labels.</t>
         </is>
       </c>
       <c r="Q5" s="5" t="n">

</xml_diff>